<commit_message>
fix: added video edit on kie
</commit_message>
<xml_diff>
--- a/public/kieVideoModelSample.xlsx
+++ b/public/kieVideoModelSample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:S9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -448,16 +448,25 @@
       <c r="P1" t="str">
         <v>pricingNote</v>
       </c>
+      <c r="Q1" t="str">
+        <v>kieInputSchema</v>
+      </c>
+      <c r="R1" t="str">
+        <v>supportsScenePreservingEdit</v>
+      </c>
+      <c r="S1" t="str">
+        <v>fixedDurations</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>OPENROUTER</v>
+        <v>KIE</v>
       </c>
       <c r="B2" t="str">
-        <v>bytedance/seedance-2.5</v>
+        <v>gemini-omni-video</v>
       </c>
       <c r="C2" t="str">
-        <v>Seedance 2.5</v>
+        <v>Gemini Omni</v>
       </c>
       <c r="D2" t="str">
         <v>GENERATE</v>
@@ -466,13 +475,13 @@
         <v>1</v>
       </c>
       <c r="F2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I2" t="b">
         <v>1</v>
@@ -480,8 +489,8 @@
       <c r="J2">
         <v>30</v>
       </c>
-      <c r="K2" t="str">
-        <v/>
+      <c r="K2">
+        <v>10</v>
       </c>
       <c r="L2" t="b">
         <v>1</v>
@@ -490,24 +499,33 @@
         <v>1</v>
       </c>
       <c r="N2" t="str">
-        <v>480p,720p</v>
+        <v>720p,1080p,4k</v>
       </c>
       <c r="O2">
-        <v>0.10387</v>
+        <v>0.07875</v>
       </c>
       <c r="P2" t="str">
-        <v>تست واقعی ۱۴۰۵/۰۶/۱۷: ۴ث/480p متن‌محض = $0.415481 -&gt; $0.1039/ث؛ فقط یک نقطه‌داده، بدون رفرنس</v>
+        <v>بدون تغییر — همون ردیف موجود، اینجا فقط برای مرجع کامل</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>OMNI</v>
+      </c>
+      <c r="R2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>OPENROUTER</v>
+        <v>KIE</v>
       </c>
       <c r="B3" t="str">
-        <v>bytedance/seedance-2.0</v>
+        <v>bytedance/seedance-2-5</v>
       </c>
       <c r="C3" t="str">
-        <v>Seedance 2.0</v>
+        <v>Seedance 2.5</v>
       </c>
       <c r="D3" t="str">
         <v>GENERATE</v>
@@ -516,7 +534,7 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -528,7 +546,7 @@
         <v>1</v>
       </c>
       <c r="J3">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="K3" t="str">
         <v/>
@@ -540,24 +558,33 @@
         <v>1</v>
       </c>
       <c r="N3" t="str">
-        <v>480p,720p,1080p,4K</v>
+        <v>480p,720p</v>
       </c>
       <c r="O3" t="str">
         <v/>
       </c>
       <c r="P3" t="str">
-        <v>تست نشده</v>
+        <v>تست نشده روی Kie (فقط روی OpenRouter تست شده بود)</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>SEEDANCE</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>OPENROUTER</v>
+        <v>KIE</v>
       </c>
       <c r="B4" t="str">
-        <v>bytedance/seedance-2.0-fast</v>
+        <v>bytedance/seedance-2</v>
       </c>
       <c r="C4" t="str">
-        <v>Seedance 2.0 Fast</v>
+        <v>Seedance 2.0</v>
       </c>
       <c r="D4" t="str">
         <v>GENERATE</v>
@@ -566,7 +593,7 @@
         <v>1</v>
       </c>
       <c r="F4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -590,24 +617,33 @@
         <v>1</v>
       </c>
       <c r="N4" t="str">
-        <v>480p,720p</v>
+        <v>480p,720p,1080p,4K</v>
       </c>
       <c r="O4" t="str">
         <v/>
       </c>
       <c r="P4" t="str">
         <v>تست نشده</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>SEEDANCE</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>OPENROUTER</v>
+        <v>KIE</v>
       </c>
       <c r="B5" t="str">
-        <v>bytedance/seedance-2.0-mini</v>
+        <v>bytedance/seedance-2-fast</v>
       </c>
       <c r="C5" t="str">
-        <v>Seedance 2.0 Mini</v>
+        <v>Seedance 2.0 Fast</v>
       </c>
       <c r="D5" t="str">
         <v>GENERATE</v>
@@ -616,7 +652,7 @@
         <v>1</v>
       </c>
       <c r="F5">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
@@ -647,17 +683,26 @@
       </c>
       <c r="P5" t="str">
         <v>تست نشده</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>SEEDANCE</v>
+      </c>
+      <c r="R5" t="b">
+        <v>0</v>
+      </c>
+      <c r="S5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>OPENROUTER</v>
+        <v>KIE</v>
       </c>
       <c r="B6" t="str">
-        <v>minimax/hailuo-3</v>
+        <v>bytedance/seedance-2-mini</v>
       </c>
       <c r="C6" t="str">
-        <v>Hailuo H3</v>
+        <v>Seedance 2.0 Mini</v>
       </c>
       <c r="D6" t="str">
         <v>GENERATE</v>
@@ -666,7 +711,7 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
@@ -690,18 +735,204 @@
         <v>1</v>
       </c>
       <c r="N6" t="str">
-        <v>2K</v>
+        <v>480p,720p</v>
       </c>
       <c r="O6" t="str">
         <v/>
       </c>
       <c r="P6" t="str">
-        <v>طبق pricing_skus رسمی: $0.13/ث پایه + $0.04 به‌ازای هر عکس رفرنس؛ تست کامل نشده</v>
+        <v>تست نشده</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>SEEDANCE</v>
+      </c>
+      <c r="R6" t="b">
+        <v>0</v>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>KIE</v>
+      </c>
+      <c r="B7" t="str">
+        <v>wan/2-6-video-to-video</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Wan 2.6 Video-to-Video</v>
+      </c>
+      <c r="D7" t="str">
+        <v>GENERATE</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>20</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7" t="b">
+        <v>0</v>
+      </c>
+      <c r="N7" t="str">
+        <v>720p,1080p</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v>تست نشده — duration فقط 5 یا 10 (enum، نه بازه)</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>WAN_V2V</v>
+      </c>
+      <c r="R7" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" t="str">
+        <v>5,10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>KIE</v>
+      </c>
+      <c r="B8" t="str">
+        <v>wan/2-7-r2v</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Wan 2.7 Reference-to-Video</v>
+      </c>
+      <c r="D8" t="str">
+        <v>GENERATE</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>21</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="b">
+        <v>1</v>
+      </c>
+      <c r="N8" t="str">
+        <v>720p,1080p</v>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v>تست نشده — duration بازه‌ی پیوسته ۲ تا ۱۰</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>WAN_R2V</v>
+      </c>
+      <c r="R8" t="b">
+        <v>0</v>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>KIE</v>
+      </c>
+      <c r="B9" t="str">
+        <v>wan/2-7-videoedit</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Wan 2.7 VideoEdit</v>
+      </c>
+      <c r="D9" t="str">
+        <v>EDIT</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>22</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>10</v>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9" t="b">
+        <v>0</v>
+      </c>
+      <c r="N9" t="str">
+        <v>720p,1080p</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v>تست نشده — تنها مدل غیر از Omni با ادیت صحنه‌حفظ‌کننده‌ی واقعی</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>WAN_VIDEO_EDIT</v>
+      </c>
+      <c r="R9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S9" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>